<commit_message>
Integrate Architecture Overview v2.1 and function papers into compliance pack
Adds Shuffle SOAR, RITA, ntopng, OpenMetadata+ELK DLP plane, PAM and
MISP to the architecture and integration diagrams; adds DXI, DLP and
XDR function figures; upgrades matrix verdicts accordingly (gaps down
from 8 to 5, now limited to mobile/MDM, email gateway and on-device
DLP control).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012XieAWwgbpjXXzkmrH6V7m
</commit_message>
<xml_diff>
--- a/jcdc-submission/JCDC_TBE-034_Praesidium_Compliance_Matrix_V2.xlsx
+++ b/jcdc-submission/JCDC_TBE-034_Praesidium_Compliance_Matrix_V2.xlsx
@@ -196,7 +196,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">36</t>
+          <t xml:space="preserve">40</t>
         </is>
       </c>
     </row>
@@ -230,7 +230,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">12</t>
+          <t xml:space="preserve">11</t>
         </is>
       </c>
     </row>
@@ -247,7 +247,7 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8</t>
+          <t xml:space="preserve">5</t>
         </is>
       </c>
     </row>
@@ -397,17 +397,17 @@
       </c>
       <c r="F3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zeek TLS fingerprinting (JA3/JA4, certificate and handshake analytics) detects malicious encrypted sessions without decryption; Wazuh correlation rules provide distributed anomaly detection across both sites</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Action for V2</t>
+          <t xml:space="preserve">ntopng Encrypted Traffic Analysis — JA3/JA3S TLS fingerprinting, SNI and certificate analytics with no session termination — plus RITA behavioural analysis (beaconing detection, DNS-tunnelling analysis, entropy scoring, C2 behaviour); Wazuh correlates across both sites for distributed anomaly detection</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comply</t>
         </is>
       </c>
       <c r="H3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V2 must name the ML analytics layer on top of Zeek metadata (anomaly-detection module trained on flow baselines). This item was answered 'Comply' in TBE-034 — the named mechanism must appear in V2 to survive material approval</t>
+          <t xml:space="preserve">Components named in Architecture Overview v2.1 — V2 plan carries the identical names so TBE-034, the overview and the plan agree</t>
         </is>
       </c>
     </row>
@@ -439,7 +439,7 @@
       </c>
       <c r="F4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wazuh behavioural rulesets (logon anomalies, process anomalies, beaconing detection) applied to Zeek network metadata and endpoint telemetry</t>
+          <t xml:space="preserve">RITA behavioural analysis over Zeek logs (beaconing, tunnelling, entropy) + Wazuh behavioural rulesets on endpoint and network telemetry</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -481,17 +481,17 @@
       </c>
       <c r="F5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zeek file-extraction framework identifies and logs file movements and types crossing monitored segments (monitor); inline control/blocking of sensitive content requires a network DLP enforcement point</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gap — decide</t>
+          <t xml:space="preserve">ntopng nDPI flow inspection (300+ application protocols) detects unauthorised uploads, tunnels and egress anomalies; ELK correlates live flows against OpenMetadata sensitivity tags (e.g. PII-tagged database exfiltrating); Shuffle SOAR enforces — perimeter block or host isolation</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comply</t>
         </is>
       </c>
       <c r="H5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Monitoring: covered. Content-aware blocking: requires a network DLP component decision or a negotiated deviation limiting scope to detect-and-alert</t>
+          <t xml:space="preserve">Control = automated containment via SOAR playbook; V2 lists the approved auto-block classes agreed with the SOC</t>
         </is>
       </c>
     </row>
@@ -607,17 +607,17 @@
       </c>
       <c r="F8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alerting real-time via Wazuh; optional blocking via Wazuh Active Response API calls to the perimeter firewalls (session teardown / ACL push)</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Action for V2</t>
+          <t xml:space="preserve">Real-time alerting via Wazuh; automated blocking via Shuffle SOAR playbooks — IP block at the perimeter firewall, host isolation, session teardown — executed in seconds without waiting on an analyst</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comply</t>
         </is>
       </c>
       <c r="H8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V2 documents the firewall-integration API (which firewall vendor CHEC deploys) and the approved auto-block rule classes</t>
+          <t xml:space="preserve">V2 documents the firewall-integration API (CHEC's firewall vendor) and the playbook catalogue</t>
         </is>
       </c>
     </row>
@@ -775,7 +775,7 @@
       </c>
       <c r="F12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wazuh Active Response (endpoint network-isolation, account disable, firewall block) orchestrated with DFIR-IRIS response workflows</t>
+          <t xml:space="preserve">Wazuh detects → DFIR-IRIS documents → Shuffle SOAR acts: predefined playbooks isolate the endpoint, block the C2 IP at the firewall, suspend the account and retrieve forensic artefacts within seconds; every action logged back to IRIS</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -785,7 +785,7 @@
       </c>
       <c r="H12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">This pairing is the SOAR answer for 272541 §1.8-O — V2 names it explicitly</t>
+          <t xml:space="preserve">This trio is the explicit SOAR answer for 272541 §1.8-O; per the integration paper, actions run in parallel with the analyst investigation</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       </c>
       <c r="F15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">MISP threat-intelligence platform (per site, replicated) feeding Wazuh CDB lists and rules; configured with JCDC-relevant use cases and watchlists per 272541 §1.8-H.7.a</t>
+          <t xml:space="preserve">MISP threat-intelligence platform (per site, replicated) feeding Wazuh CDB lists and rules; Shuffle playbooks enrich alerts from TI platforms; DXI honeynet option captures full kill-chain TTPs/IOCs for empirical, project-specific intelligence</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
@@ -911,7 +911,7 @@
       </c>
       <c r="H15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">MISP must be added to the bill of materials in V2 — the spec explicitly requires a deployed intelligence platform</t>
+          <t xml:space="preserve">MISP formally added to the V2 bill of materials — the spec requires a deployed intelligence platform with JCDC use cases and watchlists (272541 §1.8-H.7.a)</t>
         </is>
       </c>
     </row>
@@ -1867,7 +1867,7 @@
       </c>
       <c r="F38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wazuh Active Response: network isolation, process kill, account disable; DXI default-deny already contains payload execution pre-incident</t>
+          <t xml:space="preserve">Shuffle SOAR playbooks (host isolation, process kill, account disable) triggered by Wazuh detections; DXI default-deny has already contained payload execution pre-incident</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
@@ -2203,7 +2203,7 @@
       </c>
       <c r="F46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wazuh Active Response automated network isolation; DXI prevents lateral-movement tooling from executing</t>
+          <t xml:space="preserve">Shuffle SOAR automated host isolation and inter-host block (no human validation needed for predefined threat categories); DXI prevents lateral-movement tooling from executing at all</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
@@ -2371,7 +2371,7 @@
       </c>
       <c r="F50" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">MISP TI platform feeding endpoint detection rules and IOC lists</t>
+          <t xml:space="preserve">MISP TI platform feeding endpoint detection rules and IOC lists; Shuffle playbooks enrich every alert with TI context; optional DXI honeynet deployment captures full kill-chains for project-specific TTP/IOC intelligence and attribution</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr">
@@ -2455,7 +2455,7 @@
       </c>
       <c r="F52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">CMC as the single policy console for all 150k endpoints; Wazuh single pane for monitoring; both HA across the two sites</t>
+          <t xml:space="preserve">CMC as the single policy console for all 150k endpoints; Wazuh as the single monitoring pane (all telemetry converges there); IRIS as the single incident record — each HA across the two sites</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr">
@@ -2465,7 +2465,7 @@
       </c>
       <c r="H52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V2 describes the two-console operating model (policy vs monitoring) and the SOC workflow between them</t>
+          <t xml:space="preserve">V2 describes the console operating model (policy / monitoring / casework) and the SOC workflow between them, per the integration paper</t>
         </is>
       </c>
     </row>
@@ -2539,17 +2539,17 @@
       </c>
       <c r="F54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">DXI blocks new/emerging executables without signatures (zero-day-resistant by default-deny); Wazuh adds rule- and anomaly-based detection</t>
-        </is>
-      </c>
-      <c r="G54" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Action for V2</t>
+          <t xml:space="preserve">DXI blocks new and emerging executables without signatures — deterministic default-deny remains effective even against AI-generated malware; Wazuh XDR behavioural baselines (users, endpoints, applications) flag deviations, with automated threat hunts across the 120-day store</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comply</t>
         </is>
       </c>
       <c r="H54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">V2 positions default-deny as meeting the intent (blocking unknown threats) and documents the complementary detection stack; if the reviewer insists on literal on-endpoint ML, record as justified deviation</t>
+          <t xml:space="preserve">Positioning per the XDR function paper: prevention by authorisation + behavioural analytics exceeds the clause's intent of catching unknown threats</t>
         </is>
       </c>
     </row>
@@ -2707,7 +2707,7 @@
       </c>
       <c r="F58" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not in current Praesidium scope (content-aware endpoint DLP)</t>
+          <t xml:space="preserve">Network-side movement fully covered (ntopng + OpenMetadata tags correlated in ELK, Shuffle enforcement); on-device movement monitored via Wazuh (removable-media and file events) — content-aware on-device control not yet named</t>
         </is>
       </c>
       <c r="G58" s="6" t="inlineStr">
@@ -2717,7 +2717,7 @@
       </c>
       <c r="H58" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Answered 'Comply'. Wazuh detects removable-media and file events (monitor) but does not do content-aware control. Add an endpoint-DLP component or negotiate deviation — items 23–26 stand or fall together</t>
+          <t xml:space="preserve">The remaining DLP gap is device-level control only (see item 26). Decide: endpoint-DLP agent addition, demarcation, or negotiated deviation scoped to on-device control</t>
         </is>
       </c>
     </row>
@@ -2749,17 +2749,17 @@
       </c>
       <c r="F59" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not in current Praesidium scope</t>
-        </is>
-      </c>
-      <c r="G59" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gap — decide</t>
+          <t xml:space="preserve">OpenMetadata automated asset discovery and classification — continuous crawlers tag PII / financial / confidential data across SQL databases, warehouses and object storage; lineage tracking maps where tagged data flows</t>
+        </is>
+      </c>
+      <c r="G59" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Action for V2</t>
         </is>
       </c>
       <c r="H59" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Part of the DLP decision (item 23)</t>
+          <t xml:space="preserve">Per the DLP function paper. V2 confirms coverage scope for unstructured file shares alongside structured repositories</t>
         </is>
       </c>
     </row>
@@ -2791,17 +2791,17 @@
       </c>
       <c r="F60" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not in current Praesidium scope</t>
-        </is>
-      </c>
-      <c r="G60" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gap — decide</t>
+          <t xml:space="preserve">OpenMetadata classification models and pattern matching scan schema, column and content patterns to assign sensitivity tags; policy violations flagged when tagged data reaches non-compliant destinations</t>
+        </is>
+      </c>
+      <c r="G60" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Action for V2</t>
         </is>
       </c>
       <c r="H60" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Part of the DLP decision (item 23)</t>
+          <t xml:space="preserve">Same scope confirmation as item 24</t>
         </is>
       </c>
     </row>
@@ -2833,7 +2833,7 @@
       </c>
       <c r="F61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not in current Praesidium scope (device control). DXI blocks unauthorised executables launched from removable media; Wazuh logs USB events</t>
+          <t xml:space="preserve">DXI blocks unauthorised executables launched from removable media; Wazuh logs USB/device events; content-aware device control (USB write / print / clipboard) not yet named</t>
         </is>
       </c>
       <c r="G61" s="6" t="inlineStr">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="H61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Part of the DLP decision (item 23) — mitigating layers exist but are not content-aware control</t>
+          <t xml:space="preserve">The one open DLP decision — endpoint device-control component, demarcation, or deviation; items 23/26 resolve together</t>
         </is>
       </c>
     </row>
@@ -2900,7 +2900,7 @@
       </c>
       <c r="D2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Praesidium consumes decrypted-traffic logs; Zeek analyses TLS metadata without decryption</t>
+          <t xml:space="preserve">Praesidium consumes decrypted-traffic logs; ntopng/Zeek analyse TLS metadata without decryption (JA3/JA3S, SNI, certificates)</t>
         </is>
       </c>
     </row>
@@ -2922,7 +2922,7 @@
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">DNS logs ingested by SIEM; MISP supplies malicious-domain watchlists</t>
+          <t xml:space="preserve">RITA performs DNS-tunnelling analysis; Zeek dns.log + MISP malicious-domain watchlists feed detection</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2944,7 @@
       </c>
       <c r="D4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Praesidium supplies its own component backups; estate-wide backup needs an owner before V2</t>
+          <t xml:space="preserve">Praesidium supplies its own component backups; estate-wide backup needs an owner before V2. DXI's execution control is itself the strongest anti-ransomware layer</t>
         </is>
       </c>
     </row>
@@ -2983,12 +2983,12 @@
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">To be assigned — currently unowned</t>
+          <t xml:space="preserve">Praesidium — PAM included in Architecture Overview v2.1 (privileged session monitoring &amp; alerts); product name and feature mapping to be stated in V2</t>
         </is>
       </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Consoles enforce MFA + RBAC; estate-wide PAM (vaulting, session recording) needs an owner before V2</t>
+          <t xml:space="preserve">PAM session alerts feed Wazuh; PAM logs correlate in IRIS casework; asset inventory provides context</t>
         </is>
       </c>
     </row>
@@ -3039,22 +3039,22 @@
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Endpoint &amp; network DLP (content-aware)</t>
+          <t xml:space="preserve">Endpoint device control (USB write / print / clipboard)</t>
         </is>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">TBE-034 items 1.1-4, 1.5-23…26</t>
+          <t xml:space="preserve">TBE-034 items 1.5-23 / 1.5-26</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">To be decided: add DLP component or negotiate deviation</t>
+          <t xml:space="preserve">To be decided: endpoint DLP/device-control component or negotiated deviation</t>
         </is>
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zeek file reconstruction + Wazuh device auditing give monitor-grade coverage; content-aware blocking requires a DLP product</t>
+          <t xml:space="preserve">Network + repository DLP now fully named (ntopng · OpenMetadata · ELK · Shuffle); only on-device content control remains open</t>
         </is>
       </c>
     </row>
@@ -3243,7 +3243,7 @@
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Confirm dual-stack support for CMC, Wazuh, Zeek, aggregators; add to SAT</t>
+          <t xml:space="preserve">Confirm dual-stack support for CMC, Wazuh, Zeek/RITA/ntopng, aggregators; add to SAT</t>
         </is>
       </c>
     </row>
@@ -3397,7 +3397,7 @@
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Extend statement to Wazuh, IRIS, MISP consoles</t>
+          <t xml:space="preserve">Extend statement to Wazuh, IRIS, Shuffle, MISP and PAM consoles</t>
         </is>
       </c>
     </row>

</xml_diff>